<commit_message>
feat(db): historico_alimentos + relatorio de desperdicio (US-12/US-13, backend)
- migração v3: tabela historico_alimentos, restrição de status_saida, índices e view vw_desperdicio_por_categoria
- DELETE /alimentos/:id agora grava histórico antes de excluir (aceita status_saida: consumido/descartado, padrão 'descartado' até o mobile implementar a tela de confirmação)
- novos endpoints GET /relatorios/desperdicio e GET /relatorios/historico
- README atualizado (modelagem, endpoints, estrutura, Sprint 2)
- Product/Sprint Backlog reconciliados: US-01/02/03 (autenticação) e US-14 marcados fora de escopo; US-09/11/12/13 realinhadas pro time de 2 pessoas; nova US-15 (testes automatizados); aba Sprint 2 formalizada no Sprint Backlog
- bug corrigido de SP como texto que zerava o total
</commit_message>
<xml_diff>
--- a/docs/ReFood_SprintBacklog.xlsx
+++ b/docs/ReFood_SprintBacklog.xlsx
@@ -9,7 +9,8 @@
   </bookViews>
   <sheets>
     <sheet name="Sprint Backlog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Cronograma" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Sprint 2" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Cronograma" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="75">
   <si>
     <t xml:space="preserve">ReFood — Sprint Backlog (1 mês)</t>
   </si>
@@ -123,6 +124,66 @@
   </si>
   <si>
     <t xml:space="preserve">TOTAL DE STORY POINTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ReFood — Sprint 2 Backlog (planejamento)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arthur Brasil · Lucas Lonardi  |  Engenharia de Software 2026  |  26 Story Points (planejado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como usuário, quero indicar se um alimento foi consumido ou descartado ao excluí-lo, para que o sistema registre isso no histórico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modal de confirmação (Consumido/Descartado) antes de excluir · Registro salvo em historico_alimentos com categoria e data · Item continua sendo removido da listagem ativa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como usuário, quero visualizar um relatório com os alimentos que mais desperdicei por categoria, para entender meu padrão de consumo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endpoint retorna totais consumido/descartado por categoria · Tela mobile exibe o resumo · Dados batem com o histórico registrado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como usuário, quero receber uma notificação no celular quando um alimento estiver perto de vencer, mesmo sem abrir o app.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notificação local agendada na data de cadastro/edição · Permissão solicitada ao usuário · Notificação cancelada/reagendada ao editar ou excluir o item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como usuário, quero uma lista de compras com sugestões automáticas de itens em falta, para repor só o que realmente preciso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lista de compras com itens manuais e sugeridos · Item sugerido automaticamente quando some do estoque · Checkbox pra marcar como comprado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como equipe, queremos testes automatizados no backend, para garantir que mudanças futuras não quebrem funcionalidades existentes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suíte Jest + Supertest cobrindo os endpoints principais · Script npm test funcional · Roda contra um banco de teste isolado (branch do Neon)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF-06</t>
   </si>
   <si>
     <t xml:space="preserve">ReFood — Cronograma do Sprint</t>
@@ -443,11 +504,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -456,7 +521,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -787,191 +852,191 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F5" s="10" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="F6" s="10" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="10" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="F8" s="10" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="9" t="n">
+      <c r="F9" s="10" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F10" s="10" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="9" t="n">
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="10" t="n">
         <f aca="false">SUM(F5:F10)</f>
         <v>23</v>
       </c>
@@ -995,100 +1060,287 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="10" t="n">
+        <f aca="false">SUM(F5:F10)</f>
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A11:E11"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
     <tabColor rgb="FF2D6A4F"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="A1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>38</v>
+      <c r="A3" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>42</v>
+      <c r="A4" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>46</v>
+      <c r="A5" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>50</v>
+      <c r="A6" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>54</v>
+      <c r="A7" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>